<commit_message>
ci(balance): Excel과 JSON 동기화 검증 추가
</commit_message>
<xml_diff>
--- a/balance/source/balance-data.xlsx
+++ b/balance/source/balance-data.xlsx
@@ -171,7 +171,7 @@
         <v>5.0</v>
       </c>
       <c r="C2" t="n" s="0">
-        <v>10.0</v>
+        <v>100.0</v>
       </c>
       <c r="D2" t="n" s="0">
         <v>0.0</v>
@@ -182,10 +182,10 @@
         <v>2.0</v>
       </c>
       <c r="B3" t="n" s="0">
-        <v>5.0</v>
+        <v>10.0</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>20.0</v>
+        <v>200.0</v>
       </c>
       <c r="D3" t="n" s="0">
         <v>0.0</v>
@@ -196,10 +196,10 @@
         <v>3.0</v>
       </c>
       <c r="B4" t="n" s="0">
-        <v>5.0</v>
+        <v>15.0</v>
       </c>
       <c r="C4" t="n" s="0">
-        <v>30.0</v>
+        <v>300.0</v>
       </c>
       <c r="D4" t="n" s="0">
         <v>0.0</v>
@@ -210,10 +210,10 @@
         <v>4.0</v>
       </c>
       <c r="B5" t="n" s="0">
-        <v>5.0</v>
+        <v>20.0</v>
       </c>
       <c r="C5" t="n" s="0">
-        <v>40.0</v>
+        <v>400.0</v>
       </c>
       <c r="D5" t="n" s="0">
         <v>0.0</v>
@@ -224,10 +224,10 @@
         <v>5.0</v>
       </c>
       <c r="B6" t="n" s="0">
-        <v>5.0</v>
+        <v>25.0</v>
       </c>
       <c r="C6" t="n" s="0">
-        <v>50.0</v>
+        <v>500.0</v>
       </c>
       <c r="D6" t="n" s="0">
         <v>0.0</v>
@@ -238,10 +238,10 @@
         <v>6.0</v>
       </c>
       <c r="B7" t="n" s="0">
-        <v>5.0</v>
+        <v>30.0</v>
       </c>
       <c r="C7" t="n" s="0">
-        <v>60.0</v>
+        <v>600.0</v>
       </c>
       <c r="D7" t="n" s="0">
         <v>0.0</v>
@@ -252,10 +252,10 @@
         <v>7.0</v>
       </c>
       <c r="B8" t="n" s="0">
-        <v>5.0</v>
+        <v>35.0</v>
       </c>
       <c r="C8" t="n" s="0">
-        <v>70.0</v>
+        <v>700.0</v>
       </c>
       <c r="D8" t="n" s="0">
         <v>0.0</v>
@@ -266,10 +266,10 @@
         <v>8.0</v>
       </c>
       <c r="B9" t="n" s="0">
-        <v>5.0</v>
+        <v>40.0</v>
       </c>
       <c r="C9" t="n" s="0">
-        <v>80.0</v>
+        <v>800.0</v>
       </c>
       <c r="D9" t="n" s="0">
         <v>0.0</v>
@@ -280,10 +280,10 @@
         <v>9.0</v>
       </c>
       <c r="B10" t="n" s="0">
-        <v>5.0</v>
+        <v>45.0</v>
       </c>
       <c r="C10" t="n" s="0">
-        <v>90.0</v>
+        <v>900.0</v>
       </c>
       <c r="D10" t="n" s="0">
         <v>0.0</v>
@@ -294,13 +294,13 @@
         <v>10.0</v>
       </c>
       <c r="B11" t="n" s="0">
-        <v>10.0</v>
+        <v>50.0</v>
       </c>
       <c r="C11" t="n" s="0">
-        <v>150.0</v>
+        <v>1000.0</v>
       </c>
       <c r="D11" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="12">
@@ -308,13 +308,13 @@
         <v>11.0</v>
       </c>
       <c r="B12" t="n" s="0">
-        <v>10.0</v>
+        <v>55.0</v>
       </c>
       <c r="C12" t="n" s="0">
-        <v>165.0</v>
+        <v>1100.0</v>
       </c>
       <c r="D12" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="13">
@@ -322,13 +322,13 @@
         <v>12.0</v>
       </c>
       <c r="B13" t="n" s="0">
-        <v>10.0</v>
+        <v>60.0</v>
       </c>
       <c r="C13" t="n" s="0">
-        <v>180.0</v>
+        <v>1200.0</v>
       </c>
       <c r="D13" t="n" s="0">
-        <v>0.0</v>
+        <v>6.0</v>
       </c>
     </row>
     <row r="14">
@@ -336,13 +336,13 @@
         <v>13.0</v>
       </c>
       <c r="B14" t="n" s="0">
-        <v>10.0</v>
+        <v>65.0</v>
       </c>
       <c r="C14" t="n" s="0">
-        <v>195.0</v>
+        <v>1300.0</v>
       </c>
       <c r="D14" t="n" s="0">
-        <v>0.0</v>
+        <v>8.0</v>
       </c>
     </row>
     <row r="15">
@@ -350,13 +350,13 @@
         <v>14.0</v>
       </c>
       <c r="B15" t="n" s="0">
+        <v>70.0</v>
+      </c>
+      <c r="C15" t="n" s="0">
+        <v>1400.0</v>
+      </c>
+      <c r="D15" t="n" s="0">
         <v>10.0</v>
-      </c>
-      <c r="C15" t="n" s="0">
-        <v>210.0</v>
-      </c>
-      <c r="D15" t="n" s="0">
-        <v>0.0</v>
       </c>
     </row>
     <row r="16">
@@ -364,13 +364,13 @@
         <v>15.0</v>
       </c>
       <c r="B16" t="n" s="0">
-        <v>10.0</v>
+        <v>75.0</v>
       </c>
       <c r="C16" t="n" s="0">
-        <v>225.0</v>
+        <v>1500.0</v>
       </c>
       <c r="D16" t="n" s="0">
-        <v>0.0</v>
+        <v>12.0</v>
       </c>
     </row>
     <row r="17">
@@ -378,13 +378,13 @@
         <v>16.0</v>
       </c>
       <c r="B17" t="n" s="0">
-        <v>10.0</v>
+        <v>80.0</v>
       </c>
       <c r="C17" t="n" s="0">
-        <v>240.0</v>
+        <v>1600.0</v>
       </c>
       <c r="D17" t="n" s="0">
-        <v>0.0</v>
+        <v>14.0</v>
       </c>
     </row>
     <row r="18">
@@ -392,13 +392,13 @@
         <v>17.0</v>
       </c>
       <c r="B18" t="n" s="0">
-        <v>10.0</v>
+        <v>85.0</v>
       </c>
       <c r="C18" t="n" s="0">
-        <v>255.0</v>
+        <v>1700.0</v>
       </c>
       <c r="D18" t="n" s="0">
-        <v>0.0</v>
+        <v>16.0</v>
       </c>
     </row>
     <row r="19">
@@ -406,13 +406,13 @@
         <v>18.0</v>
       </c>
       <c r="B19" t="n" s="0">
-        <v>10.0</v>
+        <v>90.0</v>
       </c>
       <c r="C19" t="n" s="0">
-        <v>270.0</v>
+        <v>1800.0</v>
       </c>
       <c r="D19" t="n" s="0">
-        <v>0.0</v>
+        <v>18.0</v>
       </c>
     </row>
     <row r="20">
@@ -420,13 +420,13 @@
         <v>19.0</v>
       </c>
       <c r="B20" t="n" s="0">
-        <v>10.0</v>
+        <v>95.0</v>
       </c>
       <c r="C20" t="n" s="0">
-        <v>285.0</v>
+        <v>1900.0</v>
       </c>
       <c r="D20" t="n" s="0">
-        <v>0.0</v>
+        <v>20.0</v>
       </c>
     </row>
     <row r="21">
@@ -434,13 +434,13 @@
         <v>20.0</v>
       </c>
       <c r="B21" t="n" s="0">
-        <v>15.0</v>
+        <v>100.0</v>
       </c>
       <c r="C21" t="n" s="0">
-        <v>400.0</v>
+        <v>2000.0</v>
       </c>
       <c r="D21" t="n" s="0">
-        <v>1.0</v>
+        <v>22.0</v>
       </c>
     </row>
     <row r="22">
@@ -448,13 +448,13 @@
         <v>21.0</v>
       </c>
       <c r="B22" t="n" s="0">
-        <v>15.0</v>
+        <v>105.0</v>
       </c>
       <c r="C22" t="n" s="0">
-        <v>420.0</v>
+        <v>2100.0</v>
       </c>
       <c r="D22" t="n" s="0">
-        <v>1.0</v>
+        <v>24.0</v>
       </c>
     </row>
     <row r="23">
@@ -462,13 +462,13 @@
         <v>22.0</v>
       </c>
       <c r="B23" t="n" s="0">
-        <v>15.0</v>
+        <v>110.0</v>
       </c>
       <c r="C23" t="n" s="0">
-        <v>440.0</v>
+        <v>2200.0</v>
       </c>
       <c r="D23" t="n" s="0">
-        <v>1.0</v>
+        <v>26.0</v>
       </c>
     </row>
     <row r="24">
@@ -476,13 +476,13 @@
         <v>23.0</v>
       </c>
       <c r="B24" t="n" s="0">
-        <v>15.0</v>
+        <v>115.0</v>
       </c>
       <c r="C24" t="n" s="0">
-        <v>460.0</v>
+        <v>2300.0</v>
       </c>
       <c r="D24" t="n" s="0">
-        <v>1.0</v>
+        <v>28.0</v>
       </c>
     </row>
     <row r="25">
@@ -490,13 +490,13 @@
         <v>24.0</v>
       </c>
       <c r="B25" t="n" s="0">
-        <v>15.0</v>
+        <v>120.0</v>
       </c>
       <c r="C25" t="n" s="0">
-        <v>480.0</v>
+        <v>2400.0</v>
       </c>
       <c r="D25" t="n" s="0">
-        <v>1.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="26">
@@ -504,13 +504,13 @@
         <v>25.0</v>
       </c>
       <c r="B26" t="n" s="0">
-        <v>15.0</v>
+        <v>125.0</v>
       </c>
       <c r="C26" t="n" s="0">
-        <v>500.0</v>
+        <v>2500.0</v>
       </c>
       <c r="D26" t="n" s="0">
-        <v>1.0</v>
+        <v>32.0</v>
       </c>
     </row>
     <row r="27">
@@ -518,13 +518,13 @@
         <v>26.0</v>
       </c>
       <c r="B27" t="n" s="0">
-        <v>15.0</v>
+        <v>130.0</v>
       </c>
       <c r="C27" t="n" s="0">
-        <v>520.0</v>
+        <v>2600.0</v>
       </c>
       <c r="D27" t="n" s="0">
-        <v>1.0</v>
+        <v>34.0</v>
       </c>
     </row>
     <row r="28">
@@ -532,13 +532,13 @@
         <v>27.0</v>
       </c>
       <c r="B28" t="n" s="0">
-        <v>15.0</v>
+        <v>135.0</v>
       </c>
       <c r="C28" t="n" s="0">
-        <v>540.0</v>
+        <v>2700.0</v>
       </c>
       <c r="D28" t="n" s="0">
-        <v>1.0</v>
+        <v>36.0</v>
       </c>
     </row>
     <row r="29">
@@ -546,13 +546,13 @@
         <v>28.0</v>
       </c>
       <c r="B29" t="n" s="0">
-        <v>15.0</v>
+        <v>140.0</v>
       </c>
       <c r="C29" t="n" s="0">
-        <v>560.0</v>
+        <v>2800.0</v>
       </c>
       <c r="D29" t="n" s="0">
-        <v>1.0</v>
+        <v>38.0</v>
       </c>
     </row>
     <row r="30">
@@ -560,13 +560,13 @@
         <v>29.0</v>
       </c>
       <c r="B30" t="n" s="0">
-        <v>15.0</v>
+        <v>145.0</v>
       </c>
       <c r="C30" t="n" s="0">
-        <v>580.0</v>
+        <v>2900.0</v>
       </c>
       <c r="D30" t="n" s="0">
-        <v>1.0</v>
+        <v>40.0</v>
       </c>
     </row>
     <row r="31">
@@ -574,13 +574,13 @@
         <v>30.0</v>
       </c>
       <c r="B31" t="n" s="0">
-        <v>20.0</v>
+        <v>150.0</v>
       </c>
       <c r="C31" t="n" s="0">
-        <v>900.0</v>
+        <v>3000.0</v>
       </c>
       <c r="D31" t="n" s="0">
-        <v>2.0</v>
+        <v>42.0</v>
       </c>
     </row>
     <row r="32">
@@ -588,13 +588,13 @@
         <v>31.0</v>
       </c>
       <c r="B32" t="n" s="0">
-        <v>20.0</v>
+        <v>155.0</v>
       </c>
       <c r="C32" t="n" s="0">
-        <v>930.0</v>
+        <v>3100.0</v>
       </c>
       <c r="D32" t="n" s="0">
-        <v>2.0</v>
+        <v>44.0</v>
       </c>
     </row>
     <row r="33">
@@ -602,13 +602,13 @@
         <v>32.0</v>
       </c>
       <c r="B33" t="n" s="0">
-        <v>20.0</v>
+        <v>160.0</v>
       </c>
       <c r="C33" t="n" s="0">
-        <v>960.0</v>
+        <v>3200.0</v>
       </c>
       <c r="D33" t="n" s="0">
-        <v>2.0</v>
+        <v>46.0</v>
       </c>
     </row>
     <row r="34">
@@ -616,13 +616,13 @@
         <v>33.0</v>
       </c>
       <c r="B34" t="n" s="0">
-        <v>20.0</v>
+        <v>165.0</v>
       </c>
       <c r="C34" t="n" s="0">
-        <v>990.0</v>
+        <v>3300.0</v>
       </c>
       <c r="D34" t="n" s="0">
-        <v>2.0</v>
+        <v>48.0</v>
       </c>
     </row>
     <row r="35">
@@ -630,13 +630,13 @@
         <v>34.0</v>
       </c>
       <c r="B35" t="n" s="0">
-        <v>20.0</v>
+        <v>170.0</v>
       </c>
       <c r="C35" t="n" s="0">
-        <v>1020.0</v>
+        <v>3400.0</v>
       </c>
       <c r="D35" t="n" s="0">
-        <v>2.0</v>
+        <v>50.0</v>
       </c>
     </row>
     <row r="36">
@@ -644,13 +644,13 @@
         <v>35.0</v>
       </c>
       <c r="B36" t="n" s="0">
-        <v>20.0</v>
+        <v>175.0</v>
       </c>
       <c r="C36" t="n" s="0">
-        <v>1050.0</v>
+        <v>3500.0</v>
       </c>
       <c r="D36" t="n" s="0">
-        <v>2.0</v>
+        <v>52.0</v>
       </c>
     </row>
     <row r="37">
@@ -658,13 +658,13 @@
         <v>36.0</v>
       </c>
       <c r="B37" t="n" s="0">
-        <v>20.0</v>
+        <v>180.0</v>
       </c>
       <c r="C37" t="n" s="0">
-        <v>1080.0</v>
+        <v>3600.0</v>
       </c>
       <c r="D37" t="n" s="0">
-        <v>2.0</v>
+        <v>54.0</v>
       </c>
     </row>
     <row r="38">
@@ -672,13 +672,13 @@
         <v>37.0</v>
       </c>
       <c r="B38" t="n" s="0">
-        <v>20.0</v>
+        <v>185.0</v>
       </c>
       <c r="C38" t="n" s="0">
-        <v>1110.0</v>
+        <v>3700.0</v>
       </c>
       <c r="D38" t="n" s="0">
-        <v>2.0</v>
+        <v>56.0</v>
       </c>
     </row>
     <row r="39">
@@ -686,13 +686,13 @@
         <v>38.0</v>
       </c>
       <c r="B39" t="n" s="0">
-        <v>20.0</v>
+        <v>190.0</v>
       </c>
       <c r="C39" t="n" s="0">
-        <v>1140.0</v>
+        <v>3800.0</v>
       </c>
       <c r="D39" t="n" s="0">
-        <v>2.0</v>
+        <v>58.0</v>
       </c>
     </row>
     <row r="40">
@@ -700,13 +700,13 @@
         <v>39.0</v>
       </c>
       <c r="B40" t="n" s="0">
-        <v>20.0</v>
+        <v>195.0</v>
       </c>
       <c r="C40" t="n" s="0">
-        <v>1170.0</v>
+        <v>3900.0</v>
       </c>
       <c r="D40" t="n" s="0">
-        <v>2.0</v>
+        <v>60.0</v>
       </c>
     </row>
     <row r="41">
@@ -714,13 +714,13 @@
         <v>40.0</v>
       </c>
       <c r="B41" t="n" s="0">
-        <v>30.0</v>
+        <v>200.0</v>
       </c>
       <c r="C41" t="n" s="0">
-        <v>1600.0</v>
+        <v>4000.0</v>
       </c>
       <c r="D41" t="n" s="0">
-        <v>3.0</v>
+        <v>62.0</v>
       </c>
     </row>
     <row r="42">
@@ -728,13 +728,13 @@
         <v>41.0</v>
       </c>
       <c r="B42" t="n" s="0">
-        <v>30.0</v>
+        <v>205.0</v>
       </c>
       <c r="C42" t="n" s="0">
-        <v>1640.0</v>
+        <v>4100.0</v>
       </c>
       <c r="D42" t="n" s="0">
-        <v>3.0</v>
+        <v>64.0</v>
       </c>
     </row>
     <row r="43">
@@ -742,13 +742,13 @@
         <v>42.0</v>
       </c>
       <c r="B43" t="n" s="0">
-        <v>30.0</v>
+        <v>210.0</v>
       </c>
       <c r="C43" t="n" s="0">
-        <v>1680.0</v>
+        <v>4200.0</v>
       </c>
       <c r="D43" t="n" s="0">
-        <v>3.0</v>
+        <v>66.0</v>
       </c>
     </row>
     <row r="44">
@@ -756,13 +756,13 @@
         <v>43.0</v>
       </c>
       <c r="B44" t="n" s="0">
-        <v>30.0</v>
+        <v>215.0</v>
       </c>
       <c r="C44" t="n" s="0">
-        <v>1720.0</v>
+        <v>4300.0</v>
       </c>
       <c r="D44" t="n" s="0">
-        <v>3.0</v>
+        <v>68.0</v>
       </c>
     </row>
     <row r="45">
@@ -770,13 +770,13 @@
         <v>44.0</v>
       </c>
       <c r="B45" t="n" s="0">
-        <v>30.0</v>
+        <v>220.0</v>
       </c>
       <c r="C45" t="n" s="0">
-        <v>1760.0</v>
+        <v>4400.0</v>
       </c>
       <c r="D45" t="n" s="0">
-        <v>3.0</v>
+        <v>70.0</v>
       </c>
     </row>
     <row r="46">
@@ -784,13 +784,13 @@
         <v>45.0</v>
       </c>
       <c r="B46" t="n" s="0">
-        <v>30.0</v>
+        <v>225.0</v>
       </c>
       <c r="C46" t="n" s="0">
-        <v>1800.0</v>
+        <v>4500.0</v>
       </c>
       <c r="D46" t="n" s="0">
-        <v>3.0</v>
+        <v>72.0</v>
       </c>
     </row>
     <row r="47">
@@ -798,13 +798,13 @@
         <v>46.0</v>
       </c>
       <c r="B47" t="n" s="0">
-        <v>30.0</v>
+        <v>230.0</v>
       </c>
       <c r="C47" t="n" s="0">
-        <v>1840.0</v>
+        <v>4600.0</v>
       </c>
       <c r="D47" t="n" s="0">
-        <v>3.0</v>
+        <v>74.0</v>
       </c>
     </row>
     <row r="48">
@@ -812,13 +812,13 @@
         <v>47.0</v>
       </c>
       <c r="B48" t="n" s="0">
-        <v>30.0</v>
+        <v>235.0</v>
       </c>
       <c r="C48" t="n" s="0">
-        <v>1880.0</v>
+        <v>4700.0</v>
       </c>
       <c r="D48" t="n" s="0">
-        <v>3.0</v>
+        <v>76.0</v>
       </c>
     </row>
     <row r="49">
@@ -826,13 +826,13 @@
         <v>48.0</v>
       </c>
       <c r="B49" t="n" s="0">
-        <v>30.0</v>
+        <v>240.0</v>
       </c>
       <c r="C49" t="n" s="0">
-        <v>1920.0</v>
+        <v>4800.0</v>
       </c>
       <c r="D49" t="n" s="0">
-        <v>3.0</v>
+        <v>78.0</v>
       </c>
     </row>
     <row r="50">
@@ -840,13 +840,13 @@
         <v>49.0</v>
       </c>
       <c r="B50" t="n" s="0">
-        <v>30.0</v>
+        <v>245.0</v>
       </c>
       <c r="C50" t="n" s="0">
-        <v>1960.0</v>
+        <v>4900.0</v>
       </c>
       <c r="D50" t="n" s="0">
-        <v>3.0</v>
+        <v>80.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
[jjsh] 7-1F-4A AlienSpec 기본 스탯 외부화 구
</commit_message>
<xml_diff>
--- a/balance/source/balance-data.xlsx
+++ b/balance/source/balance-data.xlsx
@@ -9,12 +9,13 @@
     <sheet name="Config" r:id="rId3" sheetId="1"/>
     <sheet name="GameReward" r:id="rId4" sheetId="2"/>
     <sheet name="AlienUpgrade" r:id="rId5" sheetId="3"/>
+    <sheet name="AlienSpec" r:id="rId6" sheetId="4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="62">
   <si>
     <t>key</t>
   </si>
@@ -44,6 +45,162 @@
   </si>
   <si>
     <t>requiredGrowthCell</t>
+  </si>
+  <si>
+    <t>alienId</t>
+  </si>
+  <si>
+    <t>name</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>grade</t>
+  </si>
+  <si>
+    <t>baseAttack</t>
+  </si>
+  <si>
+    <t>baseMp</t>
+  </si>
+  <si>
+    <t>attackSpeed</t>
+  </si>
+  <si>
+    <t>attackRange</t>
+  </si>
+  <si>
+    <t>evolutionTargetId</t>
+  </si>
+  <si>
+    <t>isLocked</t>
+  </si>
+  <si>
+    <t>LEGEND 1</t>
+  </si>
+  <si>
+    <t>LEGEND 등급의 강력한 왹져입니다.</t>
+  </si>
+  <si>
+    <t>LEGEND</t>
+  </si>
+  <si>
+    <t>LEGEND 2</t>
+  </si>
+  <si>
+    <t>LEGEND 3</t>
+  </si>
+  <si>
+    <t>LEGEND 4</t>
+  </si>
+  <si>
+    <t>LEGEND 5</t>
+  </si>
+  <si>
+    <t>LEGEND 6</t>
+  </si>
+  <si>
+    <t>LEGEND 7</t>
+  </si>
+  <si>
+    <t>UNIQUE 1</t>
+  </si>
+  <si>
+    <t>UNIQUE 등급의 강력한 왹져입니다.</t>
+  </si>
+  <si>
+    <t>UNIQUE</t>
+  </si>
+  <si>
+    <t>UNIQUE 2</t>
+  </si>
+  <si>
+    <t>UNIQUE 3</t>
+  </si>
+  <si>
+    <t>UNIQUE 4</t>
+  </si>
+  <si>
+    <t>UNIQUE 5</t>
+  </si>
+  <si>
+    <t>UNIQUE 6</t>
+  </si>
+  <si>
+    <t>UNIQUE 7</t>
+  </si>
+  <si>
+    <t>EPIC 1</t>
+  </si>
+  <si>
+    <t>EPIC 등급의 강력한 왹져입니다.</t>
+  </si>
+  <si>
+    <t>EPIC</t>
+  </si>
+  <si>
+    <t>EPIC 2</t>
+  </si>
+  <si>
+    <t>EPIC 3</t>
+  </si>
+  <si>
+    <t>EPIC 4</t>
+  </si>
+  <si>
+    <t>EPIC 5</t>
+  </si>
+  <si>
+    <t>EPIC 6</t>
+  </si>
+  <si>
+    <t>EPIC 7</t>
+  </si>
+  <si>
+    <t>NORMAL 1</t>
+  </si>
+  <si>
+    <t>NORMAL 등급의 강력한 왹져입니다.</t>
+  </si>
+  <si>
+    <t>NORMAL</t>
+  </si>
+  <si>
+    <t>NORMAL 2</t>
+  </si>
+  <si>
+    <t>NORMAL 3</t>
+  </si>
+  <si>
+    <t>NORMAL 4</t>
+  </si>
+  <si>
+    <t>NORMAL 5</t>
+  </si>
+  <si>
+    <t>NORMAL 6</t>
+  </si>
+  <si>
+    <t>NORMAL 7</t>
+  </si>
+  <si>
+    <t>MYTHIC 1</t>
+  </si>
+  <si>
+    <t>MYTHIC 등급의 강력한 왹져입니다.</t>
+  </si>
+  <si>
+    <t>MYTHIC</t>
+  </si>
+  <si>
+    <t>MYTHIC 2</t>
+  </si>
+  <si>
+    <t>MYTHIC 3</t>
+  </si>
+  <si>
+    <t>MYTHIC 4</t>
   </si>
 </sst>
 </file>
@@ -852,4 +1009,1048 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:J33"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="J1" t="s" s="0">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E2" t="n" s="0">
+        <v>50.0</v>
+      </c>
+      <c r="F2" t="n" s="0">
+        <v>500.0</v>
+      </c>
+      <c r="G2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H2" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I2" s="0"/>
+      <c r="J2" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E3" t="n" s="0">
+        <v>50.0</v>
+      </c>
+      <c r="F3" t="n" s="0">
+        <v>500.0</v>
+      </c>
+      <c r="G3" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H3" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I3" s="0"/>
+      <c r="J3" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E4" t="n" s="0">
+        <v>50.0</v>
+      </c>
+      <c r="F4" t="n" s="0">
+        <v>500.0</v>
+      </c>
+      <c r="G4" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H4" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I4" s="0"/>
+      <c r="J4" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E5" t="n" s="0">
+        <v>50.0</v>
+      </c>
+      <c r="F5" t="n" s="0">
+        <v>500.0</v>
+      </c>
+      <c r="G5" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H5" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I5" s="0"/>
+      <c r="J5" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E6" t="n" s="0">
+        <v>50.0</v>
+      </c>
+      <c r="F6" t="n" s="0">
+        <v>500.0</v>
+      </c>
+      <c r="G6" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H6" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I6" s="0"/>
+      <c r="J6" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E7" t="n" s="0">
+        <v>50.0</v>
+      </c>
+      <c r="F7" t="n" s="0">
+        <v>500.0</v>
+      </c>
+      <c r="G7" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H7" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I7" s="0"/>
+      <c r="J7" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n" s="0">
+        <v>7.0</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E8" t="n" s="0">
+        <v>50.0</v>
+      </c>
+      <c r="F8" t="n" s="0">
+        <v>500.0</v>
+      </c>
+      <c r="G8" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H8" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I8" s="0"/>
+      <c r="J8" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E9" t="n" s="0">
+        <v>25.0</v>
+      </c>
+      <c r="F9" t="n" s="0">
+        <v>250.0</v>
+      </c>
+      <c r="G9" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H9" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I9" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="J9" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n" s="0">
+        <v>9.0</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E10" t="n" s="0">
+        <v>25.0</v>
+      </c>
+      <c r="F10" t="n" s="0">
+        <v>250.0</v>
+      </c>
+      <c r="G10" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H10" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I10" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="J10" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E11" t="n" s="0">
+        <v>25.0</v>
+      </c>
+      <c r="F11" t="n" s="0">
+        <v>250.0</v>
+      </c>
+      <c r="G11" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H11" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I11" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="J11" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n" s="0">
+        <v>11.0</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E12" t="n" s="0">
+        <v>25.0</v>
+      </c>
+      <c r="F12" t="n" s="0">
+        <v>250.0</v>
+      </c>
+      <c r="G12" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H12" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I12" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="J12" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n" s="0">
+        <v>12.0</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E13" t="n" s="0">
+        <v>25.0</v>
+      </c>
+      <c r="F13" t="n" s="0">
+        <v>250.0</v>
+      </c>
+      <c r="G13" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H13" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I13" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="J13" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E14" t="n" s="0">
+        <v>25.0</v>
+      </c>
+      <c r="F14" t="n" s="0">
+        <v>250.0</v>
+      </c>
+      <c r="G14" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H14" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I14" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="J14" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n" s="0">
+        <v>14.0</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E15" t="n" s="0">
+        <v>25.0</v>
+      </c>
+      <c r="F15" t="n" s="0">
+        <v>250.0</v>
+      </c>
+      <c r="G15" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H15" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I15" t="n" s="0">
+        <v>7.0</v>
+      </c>
+      <c r="J15" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E16" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="F16" t="n" s="0">
+        <v>150.0</v>
+      </c>
+      <c r="G16" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H16" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I16" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="J16" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n" s="0">
+        <v>16.0</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E17" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="F17" t="n" s="0">
+        <v>150.0</v>
+      </c>
+      <c r="G17" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H17" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I17" t="n" s="0">
+        <v>9.0</v>
+      </c>
+      <c r="J17" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n" s="0">
+        <v>17.0</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E18" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="F18" t="n" s="0">
+        <v>150.0</v>
+      </c>
+      <c r="G18" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H18" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I18" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="J18" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n" s="0">
+        <v>18.0</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E19" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="F19" t="n" s="0">
+        <v>150.0</v>
+      </c>
+      <c r="G19" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H19" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I19" t="n" s="0">
+        <v>11.0</v>
+      </c>
+      <c r="J19" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E20" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="F20" t="n" s="0">
+        <v>150.0</v>
+      </c>
+      <c r="G20" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H20" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I20" t="n" s="0">
+        <v>12.0</v>
+      </c>
+      <c r="J20" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n" s="0">
+        <v>20.0</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E21" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="F21" t="n" s="0">
+        <v>150.0</v>
+      </c>
+      <c r="G21" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H21" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I21" t="n" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="J21" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n" s="0">
+        <v>21.0</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C22" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="D22" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E22" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="F22" t="n" s="0">
+        <v>150.0</v>
+      </c>
+      <c r="G22" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H22" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I22" t="n" s="0">
+        <v>14.0</v>
+      </c>
+      <c r="J22" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n" s="0">
+        <v>22.0</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="C23" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="D23" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="E23" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="F23" t="n" s="0">
+        <v>100.0</v>
+      </c>
+      <c r="G23" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H23" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I23" t="n" s="0">
+        <v>15.0</v>
+      </c>
+      <c r="J23" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n" s="0">
+        <v>23.0</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C24" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="D24" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="E24" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="F24" t="n" s="0">
+        <v>100.0</v>
+      </c>
+      <c r="G24" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H24" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I24" t="n" s="0">
+        <v>16.0</v>
+      </c>
+      <c r="J24" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n" s="0">
+        <v>24.0</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="C25" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="D25" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="E25" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="F25" t="n" s="0">
+        <v>100.0</v>
+      </c>
+      <c r="G25" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H25" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I25" t="n" s="0">
+        <v>17.0</v>
+      </c>
+      <c r="J25" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n" s="0">
+        <v>25.0</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="C26" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="D26" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="E26" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="F26" t="n" s="0">
+        <v>100.0</v>
+      </c>
+      <c r="G26" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H26" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I26" t="n" s="0">
+        <v>18.0</v>
+      </c>
+      <c r="J26" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n" s="0">
+        <v>26.0</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="C27" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="D27" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="E27" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="F27" t="n" s="0">
+        <v>100.0</v>
+      </c>
+      <c r="G27" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H27" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I27" t="n" s="0">
+        <v>19.0</v>
+      </c>
+      <c r="J27" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n" s="0">
+        <v>27.0</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="C28" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="D28" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="E28" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="F28" t="n" s="0">
+        <v>100.0</v>
+      </c>
+      <c r="G28" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H28" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I28" t="n" s="0">
+        <v>20.0</v>
+      </c>
+      <c r="J28" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n" s="0">
+        <v>28.0</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C29" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="D29" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="E29" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="F29" t="n" s="0">
+        <v>100.0</v>
+      </c>
+      <c r="G29" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H29" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I29" t="n" s="0">
+        <v>21.0</v>
+      </c>
+      <c r="J29" t="b" s="0">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n" s="0">
+        <v>29.0</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="C30" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="D30" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="E30" t="n" s="0">
+        <v>100.0</v>
+      </c>
+      <c r="F30" t="n" s="0">
+        <v>1000.0</v>
+      </c>
+      <c r="G30" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H30" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I30" s="0"/>
+      <c r="J30" t="b" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n" s="0">
+        <v>30.0</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="C31" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="D31" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="E31" t="n" s="0">
+        <v>100.0</v>
+      </c>
+      <c r="F31" t="n" s="0">
+        <v>1000.0</v>
+      </c>
+      <c r="G31" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H31" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I31" s="0"/>
+      <c r="J31" t="b" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n" s="0">
+        <v>31.0</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C32" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="D32" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="E32" t="n" s="0">
+        <v>100.0</v>
+      </c>
+      <c r="F32" t="n" s="0">
+        <v>1000.0</v>
+      </c>
+      <c r="G32" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H32" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I32" s="0"/>
+      <c r="J32" t="b" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n" s="0">
+        <v>32.0</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="C33" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="D33" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="E33" t="n" s="0">
+        <v>100.0</v>
+      </c>
+      <c r="F33" t="n" s="0">
+        <v>1000.0</v>
+      </c>
+      <c r="G33" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H33" t="n" s="0">
+        <v>3.5</v>
+      </c>
+      <c r="I33" s="0"/>
+      <c r="J33" t="b" s="0">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(balance): 상점 가챠 Excel 변환과 CI 동기화 추가
</commit_message>
<xml_diff>
--- a/balance/source/balance-data.xlsx
+++ b/balance/source/balance-data.xlsx
@@ -10,12 +10,14 @@
     <sheet name="GameReward" r:id="rId4" sheetId="2"/>
     <sheet name="AlienUpgrade" r:id="rId5" sheetId="3"/>
     <sheet name="AlienSpec" r:id="rId6" sheetId="4"/>
+    <sheet name="ShopProduct" r:id="rId7" sheetId="5"/>
+    <sheet name="GachaPool" r:id="rId8" sheetId="6"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="85">
   <si>
     <t>key</t>
   </si>
@@ -201,6 +203,75 @@
   </si>
   <si>
     <t>MYTHIC 4</t>
+  </si>
+  <si>
+    <t>productId</t>
+  </si>
+  <si>
+    <t>currencyType</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>drawCount</t>
+  </si>
+  <si>
+    <t>gachaPoolId</t>
+  </si>
+  <si>
+    <t>active</t>
+  </si>
+  <si>
+    <t>ALIEN_GACHA_SINGLE</t>
+  </si>
+  <si>
+    <t>왹져 1회 뽑기</t>
+  </si>
+  <si>
+    <t>DIAMOND</t>
+  </si>
+  <si>
+    <t>STANDARD_ALIEN_POOL</t>
+  </si>
+  <si>
+    <t>ALIEN_GACHA_TEN</t>
+  </si>
+  <si>
+    <t>왹져 10회 연속 뽑기</t>
+  </si>
+  <si>
+    <t>poolId</t>
+  </si>
+  <si>
+    <t>poolName</t>
+  </si>
+  <si>
+    <t>poolActive</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>alienIds</t>
+  </si>
+  <si>
+    <t>일반 왹져 소환</t>
+  </si>
+  <si>
+    <t>22,23,24,25,26,27,28</t>
+  </si>
+  <si>
+    <t>15,16,17,18,19,20,21</t>
+  </si>
+  <si>
+    <t>8,9,10,11,12,13,14</t>
+  </si>
+  <si>
+    <t>1,2,3,4,5,6,7</t>
+  </si>
+  <si>
+    <t>29,30,31,32</t>
   </si>
 </sst>
 </file>
@@ -2053,4 +2124,213 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>66</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="D2" t="n" s="0">
+        <v>500.0</v>
+      </c>
+      <c r="E2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="G2" t="b" s="0">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>73</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="D3" t="n" s="0">
+        <v>5000.0</v>
+      </c>
+      <c r="E3" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="G3" t="b" s="0">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:F6"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C2" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="E2" t="n" s="0">
+        <v>6000.0</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C3" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E3" t="n" s="0">
+        <v>2800.0</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C4" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E4" t="n" s="0">
+        <v>900.0</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C5" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E5" t="n" s="0">
+        <v>250.0</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="C6" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="E6" t="n" s="0">
+        <v>50.0</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>84</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat(balance): 공용 보스 Lane 스폰 계약 추가
</commit_message>
<xml_diff>
--- a/balance/source/balance-data.xlsx
+++ b/balance/source/balance-data.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameReward" sheetId="2" r:id="Ra288a389c45b46ae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienSpec" sheetId="4" r:id="Ra7301815bb974dcb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopProduct" sheetId="5" r:id="R07287466c5fc47a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GachaPool" sheetId="6" r:id="Rfd9ab43137924ed3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienUpgradeCost" sheetId="7" r:id="Rad80e8e0cfff4412"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienLevelStat" sheetId="8" r:id="Rcf4fa68c1c7c4792"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpec" sheetId="9" r:id="R9990c8a81f184db0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WaveSpec" sheetId="10" r:id="R61aa011dd85b41bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WaveSpawn" sheetId="11" r:id="Rbac3bdfdf8de4faa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldLimitBalance" sheetId="12" r:id="R131e8aee660143fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SummonBalance" sheetId="13" r:id="Ra564ff342848498b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MergeRule" sheetId="14" r:id="R7955defd62114a8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicChoiceBalance" sheetId="15" r:id="R8fea9b0c63504d3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GameReward" sheetId="2" r:id="R3153ae779b45407a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienSpec" sheetId="4" r:id="R19d624c3f3894fe8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ShopProduct" sheetId="5" r:id="Rb523f60aa88b4d31"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GachaPool" sheetId="6" r:id="R96a97c75a2664393"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienUpgradeCost" sheetId="7" r:id="R2d5547afeb0f4ffa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AlienLevelStat" sheetId="8" r:id="R0c76181f0f614cd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonsterSpec" sheetId="9" r:id="R6f4765bf5ac44495"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WaveSpec" sheetId="10" r:id="Rb817b1c31418414c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WaveSpawn" sheetId="11" r:id="Refa36199e3b1496b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FieldLimitBalance" sheetId="12" r:id="R81cf21f4820146ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SummonBalance" sheetId="13" r:id="R7d4240beb4d74584"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MergeRule" sheetId="14" r:id="Ra1c9ed527a77460b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MythicChoiceBalance" sheetId="15" r:id="R72628e842292402d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5243,7 +5243,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="G13" s="38" t="str">
-        <x:v>EACH_FIELD</x:v>
+        <x:v>BOSS_SHARED</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>